<commit_message>
update the Step File
</commit_message>
<xml_diff>
--- a/Document/SMPS Design/Quatation/SMPS Price.xlsx
+++ b/Document/SMPS Design/Quatation/SMPS Price.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Open_PLCSTM32\Open_STMPLC\Document\SMPS Design\Quatation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AD04E4-065E-4440-8FF1-0BA4DB6B9AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DAF29E-C17E-43BC-918D-A22A288CC3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{E1AE2D84-7EA0-4B90-9184-4BD7CF49F92C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Sr No</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Transfomer Control &amp; Design</t>
+  </si>
+  <si>
+    <t>Shippng Charge Extra</t>
   </si>
 </sst>
 </file>
@@ -160,10 +163,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -175,10 +178,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C4C141-3E4A-4C27-81AA-657606BB96D3}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="41.7109375" bestFit="1" customWidth="1"/>
@@ -527,46 +530,41 @@
       <c r="C1" s="6"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="3">
-        <v>950</v>
-      </c>
-      <c r="C4" s="3">
+      <c r="B4" s="2">
+        <v>260</v>
+      </c>
+      <c r="C4" s="2">
         <v>1200</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
@@ -574,38 +572,47 @@
       <c r="C8" s="1"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+      <c r="A14" s="2">
         <v>1</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="3"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+      <c r="A15" s="2">
         <v>2</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="3"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+      <c r="A16" s="2">
         <v>3</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="3"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
+        <v>4</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>